<commit_message>
Analyse and update local codebase
</commit_message>
<xml_diff>
--- a/output/TSLA_Option_Valuation_Results.xlsx
+++ b/output/TSLA_Option_Valuation_Results.xlsx
@@ -9,6 +9,8 @@
   <sheets>
     <sheet name="Valuation Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Sensitivity Analysis" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="LSM Put Regressions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="LSM Call Regressions" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -991,4 +993,1352 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Time Step (t)</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Time (Years)</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>ITM Path Count</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Beta_0 (L0)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Beta_1 (L1)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Beta_2 (L2)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Beta_3 (L3)</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Exercised Paths</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Avg Continuation ($)</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Avg Imm Exercise ($)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B2" t="n">
+        <v>0.475</v>
+      </c>
+      <c r="C2" t="n">
+        <v>530</v>
+      </c>
+      <c r="D2" t="n">
+        <v>961.9881097674663</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-3296.509618473997</v>
+      </c>
+      <c r="F2" t="n">
+        <v>4487.864300787895</v>
+      </c>
+      <c r="G2" t="n">
+        <v>-1930.132704960338</v>
+      </c>
+      <c r="H2" t="n">
+        <v>349</v>
+      </c>
+      <c r="I2" t="n">
+        <v>66.3040886295816</v>
+      </c>
+      <c r="J2" t="n">
+        <v>66.85276773228192</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B3" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="C3" t="n">
+        <v>533</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1003.856452999283</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-3400.021940671334</v>
+      </c>
+      <c r="F3" t="n">
+        <v>4557.597708367847</v>
+      </c>
+      <c r="G3" t="n">
+        <v>-1928.967714140696</v>
+      </c>
+      <c r="H3" t="n">
+        <v>321</v>
+      </c>
+      <c r="I3" t="n">
+        <v>65.98347257725372</v>
+      </c>
+      <c r="J3" t="n">
+        <v>64.95764008115543</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>17</v>
+      </c>
+      <c r="B4" t="n">
+        <v>0.425</v>
+      </c>
+      <c r="C4" t="n">
+        <v>536</v>
+      </c>
+      <c r="D4" t="n">
+        <v>549.6980767618911</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-1652.07877211227</v>
+      </c>
+      <c r="F4" t="n">
+        <v>2339.741119389759</v>
+      </c>
+      <c r="G4" t="n">
+        <v>-949.7822619899282</v>
+      </c>
+      <c r="H4" t="n">
+        <v>203</v>
+      </c>
+      <c r="I4" t="n">
+        <v>65.63033268417311</v>
+      </c>
+      <c r="J4" t="n">
+        <v>62.78464758686432</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>16</v>
+      </c>
+      <c r="B5" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C5" t="n">
+        <v>552</v>
+      </c>
+      <c r="D5" t="n">
+        <v>642.103014266859</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-1960.842273934236</v>
+      </c>
+      <c r="F5" t="n">
+        <v>2689.346439204029</v>
+      </c>
+      <c r="G5" t="n">
+        <v>-1076.342418934443</v>
+      </c>
+      <c r="H5" t="n">
+        <v>240</v>
+      </c>
+      <c r="I5" t="n">
+        <v>63.59143373760304</v>
+      </c>
+      <c r="J5" t="n">
+        <v>60.56138555599266</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>15</v>
+      </c>
+      <c r="B6" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="C6" t="n">
+        <v>543</v>
+      </c>
+      <c r="D6" t="n">
+        <v>-597.6042491889558</v>
+      </c>
+      <c r="E6" t="n">
+        <v>2720.938954889014</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-3158.172935993445</v>
+      </c>
+      <c r="G6" t="n">
+        <v>1457.1382877041</v>
+      </c>
+      <c r="H6" t="n">
+        <v>117</v>
+      </c>
+      <c r="I6" t="n">
+        <v>64.59347311299048</v>
+      </c>
+      <c r="J6" t="n">
+        <v>60.63339354774038</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>14</v>
+      </c>
+      <c r="B7" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="C7" t="n">
+        <v>523</v>
+      </c>
+      <c r="D7" t="n">
+        <v>491.0662768731689</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-1322.815338765421</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1835.711060002697</v>
+      </c>
+      <c r="G7" t="n">
+        <v>-669.7198634252245</v>
+      </c>
+      <c r="H7" t="n">
+        <v>134</v>
+      </c>
+      <c r="I7" t="n">
+        <v>65.58613871587787</v>
+      </c>
+      <c r="J7" t="n">
+        <v>60.51952169354851</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>13</v>
+      </c>
+      <c r="B8" t="n">
+        <v>0.325</v>
+      </c>
+      <c r="C8" t="n">
+        <v>520</v>
+      </c>
+      <c r="D8" t="n">
+        <v>908.8731442644855</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-2818.687514210016</v>
+      </c>
+      <c r="F8" t="n">
+        <v>3659.164514978273</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-1418.228410151712</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="n">
+        <v>65.25274135887808</v>
+      </c>
+      <c r="J8" t="n">
+        <v>57.21722605800407</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>12</v>
+      </c>
+      <c r="B9" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C9" t="n">
+        <v>504</v>
+      </c>
+      <c r="D9" t="n">
+        <v>2570.478417350654</v>
+      </c>
+      <c r="E9" t="n">
+        <v>-9279.124470845751</v>
+      </c>
+      <c r="F9" t="n">
+        <v>11881.00852367958</v>
+      </c>
+      <c r="G9" t="n">
+        <v>-5097.070822346016</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>64.92276322166326</v>
+      </c>
+      <c r="J9" t="n">
+        <v>56.47689546233039</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>11</v>
+      </c>
+      <c r="B10" t="n">
+        <v>0.275</v>
+      </c>
+      <c r="C10" t="n">
+        <v>516</v>
+      </c>
+      <c r="D10" t="n">
+        <v>2168.246632940808</v>
+      </c>
+      <c r="E10" t="n">
+        <v>-7766.267073651298</v>
+      </c>
+      <c r="F10" t="n">
+        <v>9978.641066414881</v>
+      </c>
+      <c r="G10" t="n">
+        <v>-4272.947330415684</v>
+      </c>
+      <c r="H10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" t="n">
+        <v>62.60434152776473</v>
+      </c>
+      <c r="J10" t="n">
+        <v>54.00958826139385</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C11" t="n">
+        <v>503</v>
+      </c>
+      <c r="D11" t="n">
+        <v>890.7240212564392</v>
+      </c>
+      <c r="E11" t="n">
+        <v>-2688.913840100776</v>
+      </c>
+      <c r="F11" t="n">
+        <v>3451.61942426153</v>
+      </c>
+      <c r="G11" t="n">
+        <v>-1291.926908879375</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>61.55731273926293</v>
+      </c>
+      <c r="J11" t="n">
+        <v>53.31942495211575</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" t="n">
+        <v>0.225</v>
+      </c>
+      <c r="C12" t="n">
+        <v>506</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1797.882476971354</v>
+      </c>
+      <c r="E12" t="n">
+        <v>-6275.687699851299</v>
+      </c>
+      <c r="F12" t="n">
+        <v>8044.004312356542</v>
+      </c>
+      <c r="G12" t="n">
+        <v>-3379.297256629667</v>
+      </c>
+      <c r="H12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" t="n">
+        <v>59.80300313684324</v>
+      </c>
+      <c r="J12" t="n">
+        <v>50.8282454219276</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>8</v>
+      </c>
+      <c r="B13" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C13" t="n">
+        <v>506</v>
+      </c>
+      <c r="D13" t="n">
+        <v>3453.230597803278</v>
+      </c>
+      <c r="E13" t="n">
+        <v>-12526.72771310913</v>
+      </c>
+      <c r="F13" t="n">
+        <v>15866.60546538782</v>
+      </c>
+      <c r="G13" t="n">
+        <v>-6776.010702389408</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" t="n">
+        <v>58.78664902592605</v>
+      </c>
+      <c r="J13" t="n">
+        <v>47.4551850811662</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>7</v>
+      </c>
+      <c r="B14" t="n">
+        <v>0.175</v>
+      </c>
+      <c r="C14" t="n">
+        <v>497</v>
+      </c>
+      <c r="D14" t="n">
+        <v>-2991.2664336956</v>
+      </c>
+      <c r="E14" t="n">
+        <v>12253.55681508697</v>
+      </c>
+      <c r="F14" t="n">
+        <v>-15442.04768628272</v>
+      </c>
+      <c r="G14" t="n">
+        <v>7069.430512986483</v>
+      </c>
+      <c r="H14" t="n">
+        <v>14</v>
+      </c>
+      <c r="I14" t="n">
+        <v>56.72257518163747</v>
+      </c>
+      <c r="J14" t="n">
+        <v>45.62536603382232</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>6</v>
+      </c>
+      <c r="B15" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C15" t="n">
+        <v>504</v>
+      </c>
+      <c r="D15" t="n">
+        <v>-4004.067337064744</v>
+      </c>
+      <c r="E15" t="n">
+        <v>16334.2862371268</v>
+      </c>
+      <c r="F15" t="n">
+        <v>-20714.34951228985</v>
+      </c>
+      <c r="G15" t="n">
+        <v>9503.864740781362</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="n">
+        <v>54.65570935655285</v>
+      </c>
+      <c r="J15" t="n">
+        <v>41.74651388341148</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>5</v>
+      </c>
+      <c r="B16" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="C16" t="n">
+        <v>520</v>
+      </c>
+      <c r="D16" t="n">
+        <v>-2317.045141177755</v>
+      </c>
+      <c r="E16" t="n">
+        <v>10110.18217281322</v>
+      </c>
+      <c r="F16" t="n">
+        <v>-13035.09675657174</v>
+      </c>
+      <c r="G16" t="n">
+        <v>6254.039621754747</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" t="n">
+        <v>54.82184967377136</v>
+      </c>
+      <c r="J16" t="n">
+        <v>37.62865690131017</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>4</v>
+      </c>
+      <c r="B17" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C17" t="n">
+        <v>521</v>
+      </c>
+      <c r="D17" t="n">
+        <v>-11812.60715527799</v>
+      </c>
+      <c r="E17" t="n">
+        <v>48509.93468912924</v>
+      </c>
+      <c r="F17" t="n">
+        <v>-62760.09061889954</v>
+      </c>
+      <c r="G17" t="n">
+        <v>29308.00703762001</v>
+      </c>
+      <c r="H17" t="n">
+        <v>28</v>
+      </c>
+      <c r="I17" t="n">
+        <v>53.43728124643063</v>
+      </c>
+      <c r="J17" t="n">
+        <v>34.24243035898441</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>3</v>
+      </c>
+      <c r="B18" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="C18" t="n">
+        <v>517</v>
+      </c>
+      <c r="D18" t="n">
+        <v>-18962.65763883662</v>
+      </c>
+      <c r="E18" t="n">
+        <v>78079.86035419161</v>
+      </c>
+      <c r="F18" t="n">
+        <v>-101317.2475008359</v>
+      </c>
+      <c r="G18" t="n">
+        <v>47507.06225580136</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" t="n">
+        <v>50.59624578537439</v>
+      </c>
+      <c r="J18" t="n">
+        <v>31.11837697444343</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>2</v>
+      </c>
+      <c r="B19" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C19" t="n">
+        <v>499</v>
+      </c>
+      <c r="D19" t="n">
+        <v>-19044.40217663052</v>
+      </c>
+      <c r="E19" t="n">
+        <v>78783.00604511471</v>
+      </c>
+      <c r="F19" t="n">
+        <v>-102361.3682765109</v>
+      </c>
+      <c r="G19" t="n">
+        <v>48167.02215250934</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" t="n">
+        <v>47.17452903829538</v>
+      </c>
+      <c r="J19" t="n">
+        <v>24.06742148524095</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>1</v>
+      </c>
+      <c r="B20" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="C20" t="n">
+        <v>490</v>
+      </c>
+      <c r="D20" t="n">
+        <v>17449.70148531471</v>
+      </c>
+      <c r="E20" t="n">
+        <v>-72546.69538210868</v>
+      </c>
+      <c r="F20" t="n">
+        <v>95078.48298297102</v>
+      </c>
+      <c r="G20" t="n">
+        <v>-45195.4269441666</v>
+      </c>
+      <c r="H20" t="n">
+        <v>6</v>
+      </c>
+      <c r="I20" t="n">
+        <v>44.4838700469575</v>
+      </c>
+      <c r="J20" t="n">
+        <v>17.50544746011444</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Time Step (t)</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Time (Years)</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>ITM Path Count</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Beta_0 (L0)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Beta_1 (L1)</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Beta_2 (L2)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Beta_3 (L3)</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Exercised Paths</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Avg Continuation ($)</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Avg Imm Exercise ($)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B2" t="n">
+        <v>0.475</v>
+      </c>
+      <c r="C2" t="n">
+        <v>470</v>
+      </c>
+      <c r="D2" t="n">
+        <v>18.46716647155975</v>
+      </c>
+      <c r="E2" t="n">
+        <v>35.7199956195216</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-453.0677087406081</v>
+      </c>
+      <c r="G2" t="n">
+        <v>355.5575849560481</v>
+      </c>
+      <c r="H2" t="n">
+        <v>245</v>
+      </c>
+      <c r="I2" t="n">
+        <v>91.92179554476068</v>
+      </c>
+      <c r="J2" t="n">
+        <v>91.44369166018924</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B3" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="C3" t="n">
+        <v>467</v>
+      </c>
+      <c r="D3" t="n">
+        <v>82.14635739183331</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-262.486204649334</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-31.25262752322341</v>
+      </c>
+      <c r="G3" t="n">
+        <v>128.1033210238309</v>
+      </c>
+      <c r="H3" t="n">
+        <v>178</v>
+      </c>
+      <c r="I3" t="n">
+        <v>92.67990292122822</v>
+      </c>
+      <c r="J3" t="n">
+        <v>89.19107000076819</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>17</v>
+      </c>
+      <c r="B4" t="n">
+        <v>0.425</v>
+      </c>
+      <c r="C4" t="n">
+        <v>464</v>
+      </c>
+      <c r="D4" t="n">
+        <v>29.62893101732937</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-140.9231248655652</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-219.6678434183235</v>
+      </c>
+      <c r="G4" t="n">
+        <v>194.5126543756695</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>91.92136783296738</v>
+      </c>
+      <c r="J4" t="n">
+        <v>86.77781377449813</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>16</v>
+      </c>
+      <c r="B5" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C5" t="n">
+        <v>448</v>
+      </c>
+      <c r="D5" t="n">
+        <v>5.465463399548083</v>
+      </c>
+      <c r="E5" t="n">
+        <v>191.8024192369753</v>
+      </c>
+      <c r="F5" t="n">
+        <v>-671.5337737426535</v>
+      </c>
+      <c r="G5" t="n">
+        <v>491.396138201644</v>
+      </c>
+      <c r="H5" t="n">
+        <v>2</v>
+      </c>
+      <c r="I5" t="n">
+        <v>92.27707013783321</v>
+      </c>
+      <c r="J5" t="n">
+        <v>86.46476626396252</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>15</v>
+      </c>
+      <c r="B6" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="C6" t="n">
+        <v>457</v>
+      </c>
+      <c r="D6" t="n">
+        <v>50.60499396404461</v>
+      </c>
+      <c r="E6" t="n">
+        <v>99.46351428279252</v>
+      </c>
+      <c r="F6" t="n">
+        <v>-530.7988268056247</v>
+      </c>
+      <c r="G6" t="n">
+        <v>447.6982395920634</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>89.32535865013493</v>
+      </c>
+      <c r="J6" t="n">
+        <v>82.72864957607732</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>14</v>
+      </c>
+      <c r="B7" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="C7" t="n">
+        <v>477</v>
+      </c>
+      <c r="D7" t="n">
+        <v>130.9597678213057</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-483.4825851030783</v>
+      </c>
+      <c r="F7" t="n">
+        <v>280.7367347663942</v>
+      </c>
+      <c r="G7" t="n">
+        <v>-40.78563792569492</v>
+      </c>
+      <c r="H7" t="n">
+        <v>74</v>
+      </c>
+      <c r="I7" t="n">
+        <v>85.08831892060577</v>
+      </c>
+      <c r="J7" t="n">
+        <v>77.8388841828871</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>13</v>
+      </c>
+      <c r="B8" t="n">
+        <v>0.325</v>
+      </c>
+      <c r="C8" t="n">
+        <v>480</v>
+      </c>
+      <c r="D8" t="n">
+        <v>344.2373673471346</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-1661.500969937471</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1929.185290429565</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-964.0435414123492</v>
+      </c>
+      <c r="H8" t="n">
+        <v>128</v>
+      </c>
+      <c r="I8" t="n">
+        <v>83.75629230919021</v>
+      </c>
+      <c r="J8" t="n">
+        <v>75.48138922195537</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>12</v>
+      </c>
+      <c r="B9" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C9" t="n">
+        <v>496</v>
+      </c>
+      <c r="D9" t="n">
+        <v>215.7822918457386</v>
+      </c>
+      <c r="E9" t="n">
+        <v>-335.571667522786</v>
+      </c>
+      <c r="F9" t="n">
+        <v>63.34537015296182</v>
+      </c>
+      <c r="G9" t="n">
+        <v>239.2044196104711</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>80.41048468461513</v>
+      </c>
+      <c r="J9" t="n">
+        <v>69.61686331957127</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>11</v>
+      </c>
+      <c r="B10" t="n">
+        <v>0.275</v>
+      </c>
+      <c r="C10" t="n">
+        <v>484</v>
+      </c>
+      <c r="D10" t="n">
+        <v>-265.5202732827177</v>
+      </c>
+      <c r="E10" t="n">
+        <v>4369.670618468203</v>
+      </c>
+      <c r="F10" t="n">
+        <v>-6437.299883884613</v>
+      </c>
+      <c r="G10" t="n">
+        <v>4364.689622623693</v>
+      </c>
+      <c r="H10" t="n">
+        <v>116</v>
+      </c>
+      <c r="I10" t="n">
+        <v>81.22307330397032</v>
+      </c>
+      <c r="J10" t="n">
+        <v>67.78455274830193</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C11" t="n">
+        <v>497</v>
+      </c>
+      <c r="D11" t="n">
+        <v>-509.6257281241377</v>
+      </c>
+      <c r="E11" t="n">
+        <v>4940.680801437583</v>
+      </c>
+      <c r="F11" t="n">
+        <v>-7238.917871866028</v>
+      </c>
+      <c r="G11" t="n">
+        <v>4609.868886340862</v>
+      </c>
+      <c r="H11" t="n">
+        <v>3</v>
+      </c>
+      <c r="I11" t="n">
+        <v>79.04567697314394</v>
+      </c>
+      <c r="J11" t="n">
+        <v>62.75439506425678</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" t="n">
+        <v>0.225</v>
+      </c>
+      <c r="C12" t="n">
+        <v>494</v>
+      </c>
+      <c r="D12" t="n">
+        <v>-56.60545537602371</v>
+      </c>
+      <c r="E12" t="n">
+        <v>694.299640166986</v>
+      </c>
+      <c r="F12" t="n">
+        <v>-1362.298011549906</v>
+      </c>
+      <c r="G12" t="n">
+        <v>896.1079546435559</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="n">
+        <v>77.81245864973472</v>
+      </c>
+      <c r="J12" t="n">
+        <v>58.83625798077311</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>8</v>
+      </c>
+      <c r="B13" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C13" t="n">
+        <v>494</v>
+      </c>
+      <c r="D13" t="n">
+        <v>389.6021014070196</v>
+      </c>
+      <c r="E13" t="n">
+        <v>-2038.347487774724</v>
+      </c>
+      <c r="F13" t="n">
+        <v>2402.919274092082</v>
+      </c>
+      <c r="G13" t="n">
+        <v>-1257.857386492993</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" t="n">
+        <v>74.90167877174856</v>
+      </c>
+      <c r="J13" t="n">
+        <v>55.12520714509685</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>7</v>
+      </c>
+      <c r="B14" t="n">
+        <v>0.175</v>
+      </c>
+      <c r="C14" t="n">
+        <v>503</v>
+      </c>
+      <c r="D14" t="n">
+        <v>92.56425697171451</v>
+      </c>
+      <c r="E14" t="n">
+        <v>-132.3148934569142</v>
+      </c>
+      <c r="F14" t="n">
+        <v>-219.82529327574</v>
+      </c>
+      <c r="G14" t="n">
+        <v>260.4418921353956</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" t="n">
+        <v>71.76453489129059</v>
+      </c>
+      <c r="J14" t="n">
+        <v>51.56803104359248</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>6</v>
+      </c>
+      <c r="B15" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C15" t="n">
+        <v>496</v>
+      </c>
+      <c r="D15" t="n">
+        <v>-1530.249773150613</v>
+      </c>
+      <c r="E15" t="n">
+        <v>10801.47967276402</v>
+      </c>
+      <c r="F15" t="n">
+        <v>-15277.72121584373</v>
+      </c>
+      <c r="G15" t="n">
+        <v>9097.846115699525</v>
+      </c>
+      <c r="H15" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" t="n">
+        <v>70.83753450239243</v>
+      </c>
+      <c r="J15" t="n">
+        <v>49.00084496154454</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>5</v>
+      </c>
+      <c r="B16" t="n">
+        <v>0.125</v>
+      </c>
+      <c r="C16" t="n">
+        <v>480</v>
+      </c>
+      <c r="D16" t="n">
+        <v>-3478.584130340254</v>
+      </c>
+      <c r="E16" t="n">
+        <v>19477.49156169706</v>
+      </c>
+      <c r="F16" t="n">
+        <v>-27005.57714804734</v>
+      </c>
+      <c r="G16" t="n">
+        <v>14976.40482873113</v>
+      </c>
+      <c r="H16" t="n">
+        <v>12</v>
+      </c>
+      <c r="I16" t="n">
+        <v>71.58180446504655</v>
+      </c>
+      <c r="J16" t="n">
+        <v>46.38480554005205</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>4</v>
+      </c>
+      <c r="B17" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C17" t="n">
+        <v>479</v>
+      </c>
+      <c r="D17" t="n">
+        <v>-2694.642936370463</v>
+      </c>
+      <c r="E17" t="n">
+        <v>15965.40029534536</v>
+      </c>
+      <c r="F17" t="n">
+        <v>-22280.48119754853</v>
+      </c>
+      <c r="G17" t="n">
+        <v>12601.97355633373</v>
+      </c>
+      <c r="H17" t="n">
+        <v>2</v>
+      </c>
+      <c r="I17" t="n">
+        <v>69.86933276386529</v>
+      </c>
+      <c r="J17" t="n">
+        <v>39.75371311270248</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>3</v>
+      </c>
+      <c r="B18" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="C18" t="n">
+        <v>483</v>
+      </c>
+      <c r="D18" t="n">
+        <v>-1431.069664865966</v>
+      </c>
+      <c r="E18" t="n">
+        <v>8064.725043852371</v>
+      </c>
+      <c r="F18" t="n">
+        <v>-11398.17738653379</v>
+      </c>
+      <c r="G18" t="n">
+        <v>6340.770812094131</v>
+      </c>
+      <c r="H18" t="n">
+        <v>1</v>
+      </c>
+      <c r="I18" t="n">
+        <v>66.29744646490148</v>
+      </c>
+      <c r="J18" t="n">
+        <v>34.0204836028453</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>2</v>
+      </c>
+      <c r="B19" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C19" t="n">
+        <v>501</v>
+      </c>
+      <c r="D19" t="n">
+        <v>-6850.997675448067</v>
+      </c>
+      <c r="E19" t="n">
+        <v>34271.86255824999</v>
+      </c>
+      <c r="F19" t="n">
+        <v>-46966.77077518054</v>
+      </c>
+      <c r="G19" t="n">
+        <v>24900.00051241849</v>
+      </c>
+      <c r="H19" t="n">
+        <v>1</v>
+      </c>
+      <c r="I19" t="n">
+        <v>61.7227451533055</v>
+      </c>
+      <c r="J19" t="n">
+        <v>27.21418457424103</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>1</v>
+      </c>
+      <c r="B20" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="C20" t="n">
+        <v>510</v>
+      </c>
+      <c r="D20" t="n">
+        <v>12201.5701592219</v>
+      </c>
+      <c r="E20" t="n">
+        <v>-63584.644088098</v>
+      </c>
+      <c r="F20" t="n">
+        <v>86077.30399790224</v>
+      </c>
+      <c r="G20" t="n">
+        <v>-46302.63272645792</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0</v>
+      </c>
+      <c r="I20" t="n">
+        <v>57.58311454300135</v>
+      </c>
+      <c r="J20" t="n">
+        <v>18.92587320037445</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>